<commit_message>
refactor(employee-salaries): added fall back with name, change sample excel
</commit_message>
<xml_diff>
--- a/public/excel/employee_salaries.xlsx
+++ b/public/excel/employee_salaries.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/zaenalalfian/Downloads/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B98235DB-DD5B-414F-8685-6178612570C4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{385438B1-B3C8-894D-85FB-626B3E6DBA98}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="29400" windowHeight="18460" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,11 +33,14 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="13">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="18">
   <si>
     <t>employee_nip</t>
   </si>
   <si>
+    <t>employee_name</t>
+  </si>
+  <si>
     <t>salary_type</t>
   </si>
   <si>
@@ -68,10 +71,22 @@
     <t>savings_name</t>
   </si>
   <si>
+    <t>Zaenal Alfian 1</t>
+  </si>
+  <si>
     <t>monthly</t>
   </si>
   <si>
-    <t>Syirkah Full</t>
+    <t>Andre Kecap</t>
+  </si>
+  <si>
+    <t>Rai Tilosava De Araujo</t>
+  </si>
+  <si>
+    <t>Rizky Purnama Sidiq</t>
+  </si>
+  <si>
+    <t>Syirkah Penuh</t>
   </si>
 </sst>
 </file>
@@ -418,23 +433,24 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:K5"/>
+  <dimension ref="A1:L5"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="14.1640625" customWidth="1"/>
-    <col min="2" max="2" width="12.83203125" customWidth="1"/>
-    <col min="3" max="3" width="12.6640625" customWidth="1"/>
-    <col min="4" max="4" width="14.83203125" customWidth="1"/>
-    <col min="5" max="5" width="15.33203125" customWidth="1"/>
-    <col min="6" max="6" width="13.33203125" customWidth="1"/>
-    <col min="7" max="7" width="20.5" customWidth="1"/>
-    <col min="8" max="8" width="22.1640625" customWidth="1"/>
-    <col min="9" max="9" width="17.33203125" customWidth="1"/>
-    <col min="10" max="10" width="17" customWidth="1"/>
-    <col min="11" max="11" width="17.83203125" customWidth="1"/>
+    <col min="1" max="1" width="16" customWidth="1"/>
+    <col min="2" max="2" width="20.33203125" customWidth="1"/>
+    <col min="3" max="3" width="12" customWidth="1"/>
+    <col min="4" max="4" width="20.6640625" customWidth="1"/>
+    <col min="5" max="5" width="15.6640625" customWidth="1"/>
+    <col min="6" max="6" width="14.5" customWidth="1"/>
+    <col min="7" max="7" width="13.5" customWidth="1"/>
+    <col min="8" max="8" width="22.33203125" customWidth="1"/>
+    <col min="9" max="9" width="23.33203125" customWidth="1"/>
+    <col min="10" max="10" width="20.1640625" customWidth="1"/>
+    <col min="11" max="11" width="19.5" customWidth="1"/>
+    <col min="12" max="12" width="16.5" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -468,144 +484,158 @@
       <c r="K1" t="s">
         <v>10</v>
       </c>
+      <c r="L1" t="s">
+        <v>11</v>
+      </c>
     </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A2">
         <v>123124234</v>
       </c>
       <c r="B2" t="s">
-        <v>11</v>
-      </c>
-      <c r="C2">
+        <v>12</v>
+      </c>
+      <c r="C2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D2">
         <v>25</v>
       </c>
-      <c r="D2">
+      <c r="E2">
         <v>4000000</v>
       </c>
-      <c r="E2">
+      <c r="F2">
         <v>15000</v>
       </c>
-      <c r="F2">
-        <v>0</v>
-      </c>
       <c r="G2">
+        <v>0</v>
+      </c>
+      <c r="H2">
         <v>500000</v>
       </c>
-      <c r="H2">
+      <c r="I2">
         <v>1000000</v>
       </c>
-      <c r="I2">
-        <v>0</v>
-      </c>
       <c r="J2">
+        <v>0</v>
+      </c>
+      <c r="K2">
         <v>7</v>
       </c>
-      <c r="K2" t="s">
-        <v>12</v>
+      <c r="L2" s="1" t="s">
+        <v>17</v>
       </c>
     </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A3">
         <v>23493247</v>
       </c>
       <c r="B3" t="s">
-        <v>11</v>
-      </c>
-      <c r="C3">
+        <v>14</v>
+      </c>
+      <c r="C3" t="s">
+        <v>13</v>
+      </c>
+      <c r="D3">
         <v>25</v>
       </c>
-      <c r="D3">
+      <c r="E3">
         <v>1000000</v>
       </c>
-      <c r="E3">
+      <c r="F3">
         <v>15000</v>
       </c>
-      <c r="F3">
-        <v>0</v>
-      </c>
       <c r="G3">
+        <v>0</v>
+      </c>
+      <c r="H3">
         <v>300000</v>
       </c>
-      <c r="H3">
+      <c r="I3">
         <v>200000</v>
       </c>
-      <c r="I3">
-        <v>0</v>
-      </c>
       <c r="J3">
+        <v>0</v>
+      </c>
+      <c r="K3">
         <v>7</v>
       </c>
-      <c r="K3" t="s">
-        <v>12</v>
+      <c r="L3" s="1" t="s">
+        <v>17</v>
       </c>
     </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A4">
         <v>24327423</v>
       </c>
       <c r="B4" t="s">
-        <v>11</v>
-      </c>
-      <c r="C4">
+        <v>15</v>
+      </c>
+      <c r="C4" t="s">
+        <v>13</v>
+      </c>
+      <c r="D4">
         <v>25</v>
       </c>
-      <c r="D4">
+      <c r="E4">
         <v>2000000</v>
       </c>
-      <c r="E4">
+      <c r="F4">
         <v>15000</v>
       </c>
-      <c r="F4">
-        <v>0</v>
-      </c>
       <c r="G4">
+        <v>0</v>
+      </c>
+      <c r="H4">
         <v>600000</v>
       </c>
-      <c r="H4">
+      <c r="I4">
         <v>400000</v>
       </c>
-      <c r="I4">
-        <v>0</v>
-      </c>
       <c r="J4">
+        <v>0</v>
+      </c>
+      <c r="K4">
         <v>7</v>
       </c>
-      <c r="K4" t="s">
-        <v>12</v>
+      <c r="L4" s="1" t="s">
+        <v>17</v>
       </c>
     </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A5">
         <v>2342423</v>
       </c>
       <c r="B5" t="s">
-        <v>11</v>
-      </c>
-      <c r="C5">
+        <v>16</v>
+      </c>
+      <c r="C5" t="s">
+        <v>13</v>
+      </c>
+      <c r="D5">
         <v>25</v>
       </c>
-      <c r="D5">
+      <c r="E5">
         <v>2000000</v>
       </c>
-      <c r="E5">
+      <c r="F5">
         <v>15000</v>
       </c>
-      <c r="F5">
-        <v>0</v>
-      </c>
       <c r="G5">
+        <v>0</v>
+      </c>
+      <c r="H5">
         <v>600000</v>
       </c>
-      <c r="H5">
+      <c r="I5">
         <v>400000</v>
       </c>
-      <c r="I5">
-        <v>0</v>
-      </c>
       <c r="J5">
+        <v>0</v>
+      </c>
+      <c r="K5">
         <v>7</v>
       </c>
-      <c r="K5" s="1"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>